<commit_message>
subscription implementations and asana fixes
</commit_message>
<xml_diff>
--- a/docs/BACKEND_LIKE_LIMITS.xlsx
+++ b/docs/BACKEND_LIKE_LIMITS.xlsx
@@ -17,10 +17,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Changes Needed'!$A$1:$F$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questions'!$A$1:$E$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Live Test'!$A$1:$E$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questions'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Live Test'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Findings'!$A$1:$D$13</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Acceptance'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Acceptance'!$A$1:$D$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'App Behaviour'!$A$1:$C$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -62,10 +62,6 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Courier New"/>
-      <sz val="10"/>
-    </font>
-    <font>
       <b val="1"/>
       <color rgb="00B91C1C"/>
       <sz val="11"/>
@@ -79,6 +75,10 @@
       <b val="1"/>
       <color rgb="00B45309"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -127,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,19 +138,28 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -518,10 +527,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B26"/>
+  <dimension ref="A1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -585,195 +594,310 @@
     <row r="8" ht="19" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
+          <t>Updated</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="19" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
           <t>Tracker</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Gaps #22 and #33 in docs/API_CHANGES_NEEDED.md</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="10" ht="49" customHeight="1">
+      <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>On Discover a user can Like, Super Like or Pass on a profile. The admin panel sets how many likes and how many super likes a user gets per day, with different numbers for free and premium users. Passing is not limited.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="34" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>Live test</t>
-        </is>
-      </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Beta, 2026-09-11, account sp3@yopmail.com: free, Spiritual profile, no swipes before the test. Its Discover deck had only two people, so the 10-swipe limit couldn't be reached.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="19" customHeight="1">
+          <t>On Discover a user can Like, Super Like or Pass on a profile. The admin panel sets how many likes and how many super likes a user gets per day, with different numbers for free and premium users. Passing was not meant to be limited, but a pass uses up a swipe, and as of 2026-09-14 the app blocks passes too once the swipes are gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>Latest live test</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-14, nons@yopmail.com: free, Non-Spiritual, beta limits of 2 swipes and 1 super like a day. Its deck had only two people, so the refusal after the swipe limit couldn't be tested.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="19" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>First live test</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11, sp3@yopmail.com: free, Spiritual, when free accounts had 10 swipes and 1 super like a day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
           <t>App side</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Implemented 2026-09-11 in DatingDiscoverScreen and src/utils/swipeLimits.ts. See the App Behaviour sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Swagger (checked 2026-09-11)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Updated 2026-09-14 in DatingDiscoverScreen, NonSpiritualEntryScreen and src/utils/swipeLimits.ts. See the App Behaviour sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Where things stand (2026-09-14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>1. The limit refusal carries an error code</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Not done — tested: still a 400 with only a message</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>2. The swipe response returns super-like counters and resetsAt</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Done — tested</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>3. GET /api/Dating/config returns the limits and today's usage</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="inlineStr">
+        <is>
+          <t>Partly done — limits yes, usage no</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>4. The swipe response, refusal and config are documented in Swagger</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Not done</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="19" customHeight="1">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>5. Test data</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Partly done — still need a free account with 3+ people in its deck, and a premium account</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="19" customHeight="1">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Passes</t>
+        </is>
+      </c>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>Decided — a pass uses up a swipe; the app blocks ✕ once the swipes are gone</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Swagger (checked 2026-09-11, unchanged on 2026-09-14)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t>Endpoint</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>What Swagger documents</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="19" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="26" ht="19" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>POST /api/Dating/swipe</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Body RecordSwipeRequest { swipedUserId: int, action: string }. Response: 200 OK only, untyped.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="19" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="27" ht="19" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>GET /api/Dating/config</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>"200 OK", untyped.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="49" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="28" ht="34" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>GET /api/admin/settings
 PUT /api/admin/settings/{key}</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Body { settingValue: string }. Setting keys aren't listed.</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Sheets in this file</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>What's in it</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="19" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
+    <row r="32" ht="19" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>Changes Needed</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B32" s="5" t="inlineStr">
         <is>
           <t>What the backend needs to build or change, with a column for backend notes.</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="19" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
+    <row r="33" ht="19" customHeight="1">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>Questions</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B33" s="5" t="inlineStr">
         <is>
           <t>Rules the backend should confirm, and product questions for the client, with an Answer column.</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="19" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
+    <row r="34" ht="19" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Live Test</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>The three swipe requests made on beta and what each returned.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="19" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>Every swipe request made on beta and what each returned.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="19" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Findings</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>What the live test shows, what is still untested, and another issue seen in the same session.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="19" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>What the live tests show, what is still untested, and another issue seen along the way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="19" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>Acceptance</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B36" s="5" t="inlineStr">
         <is>
           <t>The checklist for signing this off.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="19" customHeight="1">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="37" ht="19" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>App Behaviour</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>What the app does now, and what it will do once the backend ships.</t>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>What the app does now, and what it will do once the rest ships.</t>
         </is>
       </c>
     </row>
@@ -799,7 +923,7 @@
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="58" customWidth="1" min="3" max="3"/>
     <col width="62" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -836,7 +960,7 @@
       </c>
     </row>
     <row r="2" ht="147" customHeight="1">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -846,11 +970,12 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Keep the message, but add a machine-readable code, and preferably use HTTP 403 as agreed with the client.
-code is SWIPE_LIMIT_REACHED (the daily 10) or SUPERLIKE_LIMIT_REACHED. Nothing else should use these codes.</t>
-        </is>
-      </c>
-      <c r="D2" s="7" t="inlineStr">
+          <t>Tested 2026-09-14: the refusal is still a 400 with only a message.
+Keep the message, but add a machine-readable code, and preferably use HTTP 403 as agreed with the client.
+code is SWIPE_LIMIT_REACHED (the daily swipes) or SUPERLIKE_LIMIT_REACHED. Nothing else should use these codes. Add the error response to Swagger.</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>HTTP 403
 {
@@ -859,20 +984,20 @@
   "data": {
     "code": "SUPERLIKE_LIMIT_REACHED",
     "limit": 1,
-    "resetsAt": "2026-09-12T00:00:00Z"
+    "resetsAt": "2026-09-15T00:00:00Z"
   }
 }</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E2" s="11" t="inlineStr">
+        <is>
+          <t>Not done</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr"/>
     </row>
-    <row r="3" ht="160" customHeight="1">
-      <c r="A3" s="6" t="n">
+    <row r="3" ht="173" customHeight="1">
+      <c r="A3" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -882,56 +1007,76 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>The swipe response already has the swipe counters. Add the super-like ones and resetsAt.</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>{
+          <t>Tested 2026-09-14: the swipe response carries dailySuperLikeLimit, superLikesUsedToday, superLikesRemainingToday and resetsAt (midnight UTC). Only the Swagger documentation is left (#4).</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
+          <t>Returned on beta 2026-09-14:
+{
   "isMatch": false,
   "matchId": null,
   "isPremium": false,
-  "dailySwipeLimit": 10,
+  "dailySwipeLimit": 2,
   "swipesUsedToday": 1,
-  "swipesRemainingToday": 9,
+  "swipesRemainingToday": 1,
   "dailySuperLikeLimit": 1,
   "superLikesUsedToday": 1,
   "superLikesRemainingToday": 0,
-  "resetsAt": "2026-09-12T00:00:00Z"
+  "resetsAt": "2026-09-15T00:00:00Z"
 }</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
-        <is>
-          <t>Open</t>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr"/>
     </row>
-    <row r="4" ht="49" customHeight="1">
-      <c r="A4" s="6" t="n">
+    <row r="4" ht="212" customHeight="1">
+      <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Return the same counters from GET /api/Dating/config</t>
+          <t>Return today's usage from GET /api/Dating/config</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Put them next to maxGalleryImages, so the app knows the limits before the first swipe. It can then show the real numbers instead of hardcoded ones and dim ♥/⭐ up front. Use null for unlimited.</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr"/>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>The limits are there (freeSwipesPerDay, freeSuperLikesPerDay, premiumSwipesPerDay, premiumSuperLikesPerDay). Add the usage fields the swipe response already has (swipesUsedToday, swipesRemainingToday, superLikesUsedToday, superLikesRemainingToday, resetsAt), so the app knows where the user stands before their first swipe of a session and can dim ♥/⭐ straight away. Use null for unlimited.</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Returned on beta 2026-09-14:
+{
+  "freeSuperLikesPerDay": 1,
+  "freeSwipesPerDay": 2,
+  "maxDatingImages": 6,
+  "maxGalleryImages": 5,
+  "maxIceBreakers": 1,
+  "otpExpiryMinutes": 10,
+  "otpLength": 6,
+  "premiumSuperLikesPerDay": 5,
+  "premiumSwipesPerDay": 2,
+  "supportEmail": "support@email.com",
+  "trialDays_DatingNonSpiritual": 3,
+  "trialDays_DatingSpiritual": 3,
+  "vettingPassScore": 10
+}</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>Partly done</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="6" t="n">
+      <c r="A5" s="9" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -941,19 +1086,19 @@
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Add the limit error response, and type the swipe response and GET /api/Dating/config, which are documented as a bare "200 OK" today.</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr"/>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>The swipe response, the limit refusal and GET /api/Dating/config are all still documented as a bare "200 OK".</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr"/>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Not done</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr"/>
     </row>
-    <row r="6" ht="79" customHeight="1">
-      <c r="A6" s="6" t="n">
+    <row r="6" ht="94" customHeight="1">
+      <c r="A6" s="9" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="5" t="inlineStr">
@@ -963,13 +1108,13 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>A premium account with a dating profile, to check the premium values.
-A deck with more than 10 people, or a temporarily lower limit on beta (e.g. 2 swipes), to test the swipe limit.
+          <t>A free account with at least 3 people in its Discover deck, to test the refusal for the swipe after the limit (sp3@yopmail.com and nons@yopmail.com have swiped everyone in theirs).
+A premium account with a dating profile, to check the premium values.
 For reference: chat.michael@yopmail.com (in CHAT_API.md) is deactivated, and sp2@yopmail.com has no dating profile.</t>
         </is>
       </c>
-      <c r="D6" s="7" t="inlineStr"/>
-      <c r="E6" s="8" t="inlineStr">
+      <c r="D6" s="10" t="inlineStr"/>
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -988,14 +1133,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="64" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1021,113 +1167,151 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
           <t>Answer</t>
         </is>
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Does a Pass count toward dailySwipeLimit?</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
+          <t>Should a Pass use up a swipe?</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>Backend + client</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Tested 2026-09-14: it does (swipesUsedToday went from 1 to 2).</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>Yes (2026-09-14). The app blocks passes once the swipes are gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Is a Pass refused once the swipes run out?</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>The requirement is that passes aren't limited, but the name "swipes" suggests they might be.</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr"/>
-    </row>
-    <row r="3" ht="19" customHeight="1">
-      <c r="A3" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>Is the 10 a limit on likes or on all swipes?</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Not tested yet. The app no longer sends one when it knows the swipes are gone, but it should get the same refusal as a like if it does.</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>When does the count reset?</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>The admin panel, the API and the app copy should use the same word.</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr"/>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>When does the count reset: midnight UTC, the user's local midnight, or a rolling 24 hours?</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>resetsAt in the swipe response.</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>Midnight UTC ("2026-09-15T00:00:00Z", tested 2026-09-14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Do Spiritual and Non-Spiritual dating share the same limits?</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Return resetsAt as UTC with a Z (see gap #30). Until then the app guesses local midnight.</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr"/>
-    </row>
-    <row r="5" ht="19" customHeight="1">
-      <c r="A5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Do Spiritual and Non-Spiritual dating share the same limits?</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Which admin setting keys hold these values, and does a change apply immediately?</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr"/>
-      <c r="E5" s="5" t="inlineStr"/>
-    </row>
-    <row r="6" ht="34" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Which admin setting keys hold these values, and does a change apply immediately?</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Backend</t>
-        </is>
-      </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
           <t>The keys for PUT /api/admin/settings/{key} aren't listed in Swagger.</t>
         </is>
       </c>
-      <c r="E6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7" ht="49" customHeight="1">
-      <c r="A7" s="6" t="n">
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+    </row>
+    <row r="7" ht="64" customHeight="1">
+      <c r="A7" s="9" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -1135,41 +1319,25 @@
           <t>Is premium ever unlimited?</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>Client</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>The Figma copy says "Unlimited Likes" (Premium screen) and "Try Premium subscription for unlimited swaps and filters" (limit cover). If premium has a cap, both need new wording.</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr"/>
-    </row>
-    <row r="8" ht="19" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Should Pass stay unlimited?</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Client</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Assumed yes.</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr"/>
+          <t>The Figma copy says "Unlimited Likes" (Premium screen) and "Try Premium subscription for unlimited swaps and filters" (limit cover). If premium has a cap, both need new wording. On beta, config currently gives premium 2 swipes and 5 super likes a day, so that wording is wrong there.</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:F7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1180,56 +1348,203 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="64" customWidth="1" min="4" max="4"/>
-    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="4" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Request</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>HTTP</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Response body</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>What it shows</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="108" customHeight="1">
-      <c r="A2" s="6" t="n">
+    <row r="2" ht="160" customHeight="1">
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>nons@yopmail.com</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>SuperLike user 73</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>{
+  "isMatch": false,
+  "matchId": null,
+  "isPremium": false,
+  "dailySwipeLimit": 2,
+  "swipesUsedToday": 1,
+  "swipesRemainingToday": 1,
+  "dailySuperLikeLimit": 1,
+  "superLikesUsedToday": 1,
+  "superLikesRemainingToday": 0,
+  "resetsAt": "2026-09-15T00:00:00Z"
+}</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>Accepted. Carries the new super-like counters and resetsAt (midnight UTC).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="82" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>nons@yopmail.com</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>SuperLike user 254</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>400</v>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
+          <t>{
+  "success": false,
+  "message": "You have reached your daily limit of 1 super likes. Upgrade to Premium for more.",
+  "errors": null
+}</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Refused: 1 super like a day. Still a 400 with no error code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="160" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>nons@yopmail.com</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Ignore user 254</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>200</v>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>{
+  "isMatch": false,
+  "matchId": null,
+  "isPremium": false,
+  "dailySwipeLimit": 2,
+  "swipesUsedToday": 2,
+  "swipesRemainingToday": 0,
+  "dailySuperLikeLimit": 1,
+  "superLikesUsedToday": 1,
+  "superLikesRemainingToday": 0,
+  "resetsAt": "2026-09-15T00:00:00Z"
+}</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>A pass uses up a swipe: swipesUsedToday went from 1 to 2. The refused super like wasn't counted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="108" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>sp3@yopmail.com</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>SuperLike user 84</t>
         </is>
       </c>
-      <c r="C2" s="9" t="n">
+      <c r="E5" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="F5" s="10" t="inlineStr">
         <is>
           <t>{
   "isMatch": false,
@@ -1241,25 +1556,35 @@
 }</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>Accepted. A super like also counts as a swipe: swipesUsedToday went from 0 to 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="82" customHeight="1">
-      <c r="A3" s="6" t="n">
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Accepted. A super like also counts as a swipe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="82" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>sp3@yopmail.com</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
         <is>
           <t>SuperLike user 189</t>
         </is>
       </c>
-      <c r="C3" s="8" t="n">
+      <c r="E6" s="11" t="n">
         <v>400</v>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="F6" s="10" t="inlineStr">
         <is>
           <t>{
   "success": false,
@@ -1268,25 +1593,35 @@
 }</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>Free accounts get 1 super like a day. The refusal is a 400 with no error code (the agreed contract was 402/403).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="108" customHeight="1">
-      <c r="A4" s="6" t="n">
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Refused: 1 super like a day. A 400 with no error code (the agreed contract was 402/403).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="108" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>sp3@yopmail.com</t>
+        </is>
+      </c>
+      <c r="C7" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Like user 189</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n">
+      <c r="E7" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="F7" s="10" t="inlineStr">
         <is>
           <t>{
   "isMatch": true,
@@ -1298,14 +1633,14 @@
 }</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>Running out of super likes doesn't block likes. The refused super like didn't count: the count only moved to 2 here.</t>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Likes still work after super likes run out. The refused super like didn't count.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E4"/>
+  <autoFilter ref="A1:G7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1322,7 +1657,7 @@
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="44" customWidth="1" min="2" max="2"/>
     <col width="80" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1348,7 +1683,7 @@
       </c>
     </row>
     <row r="2" ht="19" customHeight="1">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1358,209 +1693,213 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>Free users get 1 super like and 10 swipes a day.</t>
-        </is>
-      </c>
-      <c r="D2" s="9" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="19" customHeight="1">
-      <c r="A3" s="6" t="n">
+          <t>A free account is refused a super like past its daily limit (both tests).</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>A super like also counts as a swipe</t>
+          <t>The swipe response carries super-like counters and resetsAt</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Live Test step 1 took swipesUsedToday from 0 to 1.</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="19" customHeight="1">
-      <c r="A4" s="6" t="n">
+          <t>dailySuperLikeLimit, superLikesUsedToday, superLikesRemainingToday and resetsAt "2026-09-15T00:00:00Z" (midnight UTC), next to the swipe counters and isPremium.</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="49" customHeight="1">
+      <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>A refused swipe doesn't count</t>
+          <t>The refusal still has no error code</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>The count only moved to 2 with the like in Live Test step 3.</t>
-        </is>
-      </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="19" customHeight="1">
-      <c r="A5" s="6" t="n">
+          <t>A 400 with only a message. The API also uses 400 for other failures (e.g. GET /api/Dating/discover answers 400 "Please set up your dating profile before discovering."), so the app has to recognise a limit by its wording.</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="9" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
+          <t>A Pass uses up a swipe</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>swipesUsedToday went from 1 to 2 on an Ignore. Decided 2026-09-14 to keep it: the app blocks passes at the limit.</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>A super like also uses up a swipe</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>swipesUsedToday rises on a super like (both tests).</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="19" customHeight="1">
+      <c r="A7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>A refused swipe isn't counted or saved</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>The count didn't move on the refusal, and GET /api/Dating/likes/sent doesn't list it.</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="19" customHeight="1">
+      <c r="A8" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
           <t>Running out of super likes doesn't block likes</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Live Test step 3.</t>
-        </is>
-      </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="49" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>The refusal is a 400 with no error code</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>The contract agreed with the client was 402/403. The API also uses 400 for other failures (e.g. GET /api/Dating/discover answers 400 "Please set up your dating profile before discovering."), so the app can only recognise a limit by the wording of message.</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>The swipe response already carries swipe counters</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>dailySwipeLimit, swipesUsedToday, swipesRemainingToday and isPremium. There's nothing for super likes, no reset time, and none of it is in Swagger.</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="19" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>The limits can't be read before swiping</t>
-        </is>
-      </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>GET /api/Dating/config returns only { "maxGalleryImages": 4 }.</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Verified</t>
+          <t>A like right after the refusal went through.</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-11</t>
         </is>
       </c>
     </row>
     <row r="9" ht="34" customHeight="1">
-      <c r="A9" s="6" t="n">
+      <c r="A9" s="9" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
+          <t>Config returns the limits, not usage</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>GET /api/Dating/config returns freeSwipesPerDay, freeSuperLikesPerDay, premiumSwipesPerDay and premiumSuperLikesPerDay (beta: 2, 1, 2, 5). On 2026-09-11 it returned only maxGalleryImages.</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
           <t>Likes Received isn't premium-gated</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>GET /api/Dating/likes/received returned the full list to this free account (200 with data). Gap #23.</t>
-        </is>
-      </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Verified</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="19" customHeight="1">
-      <c r="A10" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>What the 11th swipe returns</t>
-        </is>
-      </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>The Discover deck had only two people.</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="inlineStr">
+          <t>GET /api/Dating/likes/received returned the full list to a free account (200 with data). Gap #23.</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="19" customHeight="1">
+      <c r="A11" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>The swipe after the daily limit is refused</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Needs an account with at least 3 people in its Discover deck.</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="19" customHeight="1">
-      <c r="A11" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Whether a Pass counts toward the 10</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="10" t="inlineStr">
+    <row r="12" ht="19" customHeight="1">
+      <c r="A12" s="9" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Whether a Pass is refused once the swipes run out</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr"/>
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="19" customHeight="1">
-      <c r="A12" s="6" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>When the count resets</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="10" t="inlineStr">
-        <is>
-          <t>Not tested</t>
-        </is>
-      </c>
-    </row>
     <row r="13" ht="19" customHeight="1">
-      <c r="A13" s="6" t="n">
+      <c r="A13" s="9" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="5" t="inlineStr">
@@ -1573,7 +1912,7 @@
           <t>Needs a premium account with a dating profile.</t>
         </is>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>Not tested</t>
         </is>
@@ -1591,7 +1930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1623,7 +1962,7 @@
       </c>
     </row>
     <row r="2" ht="34" customHeight="1">
-      <c r="A2" s="6" t="n">
+      <c r="A2" s="9" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1631,19 +1970,19 @@
           <t>Free user: the 2nd super like of the day is refused, and likes still work afterwards.</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="C2" s="12" t="inlineStr">
         <is>
           <t>Verified 2026-09-11</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>sp3@yopmail.com, Live Test steps 2–3.</t>
+          <t>sp3@yopmail.com</t>
         </is>
       </c>
     </row>
     <row r="3" ht="19" customHeight="1">
-      <c r="A3" s="6" t="n">
+      <c r="A3" s="9" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -1651,131 +1990,151 @@
           <t>A refused swipe doesn't use up allowance.</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Verified 2026-09-11</t>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Live Test steps 1–3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="34" customHeight="1">
-      <c r="A4" s="6" t="n">
+          <t>Also seen on 2026-09-11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="19" customHeight="1">
+      <c r="A4" s="9" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Free user: the 11th swipe is refused with SWIPE_LIMIT_REACHED.</t>
-        </is>
-      </c>
-      <c r="C4" s="10" t="inlineStr">
+          <t>GET /api/Dating/config returns the free and premium limits.</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr"/>
+    </row>
+    <row r="5" ht="19" customHeight="1">
+      <c r="A5" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>The swipe response carries super-like counters and resetsAt.</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Verified 2026-09-14</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr"/>
+    </row>
+    <row r="6" ht="19" customHeight="1">
+      <c r="A6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Refusals carry a code and are documented in Swagger.</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>Needs a deck with more than 10 people, or a lower limit on beta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="19" customHeight="1">
-      <c r="A5" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Refusals carry a code and are documented in Swagger.</t>
-        </is>
-      </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Changes Needed #1 and #4. Tested 2026-09-14: no code yet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Free user: the swipe after the daily limit is refused with SWIPE_LIMIT_REACHED.</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>Changes Needed #1 and #4.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="19" customHeight="1">
-      <c r="A6" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>A Pass is never refused for a limit.</t>
-        </is>
-      </c>
-      <c r="C6" s="10" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Needs an account with at least 3 people in its Discover deck.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="19" customHeight="1">
+      <c r="A8" s="9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>A pass after the daily limit is refused the same way as a like.</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
-    </row>
-    <row r="7" ht="19" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>That a pass uses up a swipe is verified (2026-09-14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="19" customHeight="1">
+      <c r="A9" s="9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>A premium user gets the premium values.</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Needs a premium account with a dating profile.</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="19" customHeight="1">
-      <c r="A8" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>The count resets when resetsAt says.</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
+    <row r="10" ht="19" customHeight="1">
+      <c r="A10" s="9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>GET /api/Dating/config includes today's usage.</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr"/>
-    </row>
-    <row r="9" ht="19" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>Limits and usage come back from the swipe response and GET /api/Dating/config.</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>Changes Needed #2 and #3.</t>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Changes Needed #3.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1789,8 +2148,8 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="96" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -1811,173 +2170,173 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="49" customHeight="1">
+    <row r="2" ht="34" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Now (2026-09-11)</t>
+          <t>Now (2026-09-14)</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>Recognising a limit</t>
+          <t>After a successful swipe</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>A refused swipe counts as "that allowance is spent" when it is a 402/403 (the agreed contract) or a 400 whose message contains "daily limit" (what the API actually sends). The wording match is a stopgap: rewording the message breaks it.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="19" customHeight="1">
+          <t>Reads the counters. No swipes left → ♥, ✕ and ⭐ are dimmed. No super likes left → ⭐ is dimmed. Some left → the block lifts. Remembers resetsAt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Now (2026-09-11)</t>
+          <t>Now (2026-09-14)</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Like refused</t>
+          <t>Before any counters arrive</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>The card goes back, the "You Have Reached Your Daily Limit!" cover shows, and ♥ is dimmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="19" customHeight="1">
+          <t>For the first swipe of a session, a refusal counts as "that allowance is spent" when it is a 402/403, or a 400 whose message contains "daily limit". The wording match is a stopgap until the error code ships.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Now (2026-09-11)</t>
+          <t>Now (2026-09-14)</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Super Like refused</t>
+          <t>Like or pass with no swipes left</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>The card goes back, an "Out of Super Likes" alert shows, and ⭐ is dimmed. Likes keep working.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="19" customHeight="1">
+          <t>The card goes back and the "You Have Reached Your Daily Limit!" cover shows. A super like does the same once the swipes are gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Now (2026-09-11)</t>
+          <t>Now (2026-09-14)</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Super Like with only super likes gone</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Never treated as limited.</t>
+          <t>The card goes back and an "Out of Super Likes" alert shows. Likes keep working.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="19" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Now (2026-09-11)</t>
+          <t>Now (2026-09-14)</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Blocked once the swipes are gone, since a pass uses up a swipe (decided 2026-09-14).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="19" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Now (2026-09-14)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
           <t>Any other failure</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Treated as transient.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="34" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Now (2026-09-11)</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Reset</t>
-        </is>
-      </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>The block lifts at the device's local midnight (a guess), or when the user buys premium. If the server hasn't reset yet, the next swipe is refused again.</t>
+          <t>The card goes back and the server's message shows in a toast (since 2026-09-15), so a readable message matters.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="34" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Now (2026-09-11)</t>
+          <t>Now (2026-09-14)</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Numbers shown</t>
+          <t>Reset</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>Hardcoded on the Non-Spiritual entry screen: "10 free swipes per day" and "1 super like per day". They match beta today, but won't follow an admin change.</t>
+          <t>The block is saved on the device, so it survives a relaunch. It lifts at the last resetsAt seen, or at the next midnight UTC without one, which matches the server. Buying premium clears limits reached on the free plan.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Once the backend ships</t>
+          <t>Now (2026-09-14)</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Recognising a limit</t>
+          <t>Numbers shown</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Read code instead of matching the message text.</t>
+          <t>The Non-Spiritual entry screen shows the free numbers from GET /api/Dating/config.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Once the backend ships</t>
+          <t>Once the rest ships</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Numbers shown</t>
+          <t>Recognising a limit</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>Load the limits on Discover focus, dim ♥/⭐ up front, and show the admin numbers on the Non-Spiritual entry screen.</t>
+          <t>Read code instead of matching the message text.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Once the backend ships</t>
+          <t>Once the rest ships</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Reset</t>
+          <t>Dimming up front</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Lift the block at resetsAt instead of local midnight.</t>
+          <t>Read today's usage from GET /api/Dating/config on Discover focus, and dim ♥/⭐ before the first swipe of a session.</t>
         </is>
       </c>
     </row>

</xml_diff>